<commit_message>
found minor error in statistical tests through GPT-OSS runs with 193 scenarios (2 fully failed scenarios)
</commit_message>
<xml_diff>
--- a/Analysis/diagnostics/significance_pooled_diagnostics_NOT_FOR_PAPER.xlsx
+++ b/Analysis/diagnostics/significance_pooled_diagnostics_NOT_FOR_PAPER.xlsx
@@ -629,13 +629,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.631034</v>
+        <v>-0.613846</v>
       </c>
       <c r="D9" t="n">
-        <v>0.022149</v>
+        <v>0.025823</v>
       </c>
       <c r="E9" t="n">
-        <v>-28.4906</v>
+        <v>-23.7716</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -653,13 +653,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-0.631116</v>
+        <v>-0.613333</v>
       </c>
       <c r="D10" t="n">
-        <v>0.023283</v>
+        <v>0.027516</v>
       </c>
       <c r="E10" t="n">
-        <v>-27.1069</v>
+        <v>-22.2903</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -677,13 +677,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.422044</v>
+        <v>-0.403846</v>
       </c>
       <c r="D11" t="n">
-        <v>0.01661</v>
+        <v>0.016822</v>
       </c>
       <c r="E11" t="n">
-        <v>-25.4086</v>
+        <v>-24.0067</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -701,13 +701,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.198732</v>
+        <v>-0.176923</v>
       </c>
       <c r="D12" t="n">
-        <v>0.016211</v>
+        <v>0.022082</v>
       </c>
       <c r="E12" t="n">
-        <v>-12.2593</v>
+        <v>-8.012</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -725,13 +725,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.115984</v>
+        <v>0.109499</v>
       </c>
       <c r="D13" t="n">
-        <v>0.006112</v>
+        <v>0.006162</v>
       </c>
       <c r="E13" t="n">
-        <v>18.9754</v>
+        <v>17.7691</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -749,13 +749,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.132714</v>
+        <v>0.125019</v>
       </c>
       <c r="D14" t="n">
-        <v>0.006868</v>
+        <v>0.004882</v>
       </c>
       <c r="E14" t="n">
-        <v>19.3222</v>
+        <v>25.6096</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -1073,10 +1073,10 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>-20.2361</v>
+        <v>-19.8976</v>
       </c>
       <c r="H9" t="n">
-        <v>4.714517838173366e-91</v>
+        <v>4.268500509053557e-88</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="b">
@@ -1103,10 +1103,10 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>-20.0999</v>
+        <v>-19.6622</v>
       </c>
       <c r="H10" t="n">
-        <v>7.388884514679244e-90</v>
+        <v>4.546037539374914e-86</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="b">
@@ -1133,10 +1133,10 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>-18.2115</v>
+        <v>-17.6995</v>
       </c>
       <c r="H11" t="n">
-        <v>4.181391047286391e-74</v>
+        <v>4.230060305968027e-70</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="b">
@@ -1163,10 +1163,10 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>-13.8335</v>
+        <v>-12.2364</v>
       </c>
       <c r="H12" t="n">
-        <v>1.60055911857265e-43</v>
+        <v>1.985791909668446e-34</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="b">
@@ -1193,10 +1193,10 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>22.4403</v>
+        <v>21.3267</v>
       </c>
       <c r="H13" t="n">
-        <v>1.591469121032303e-111</v>
+        <v>6.416330059507789e-101</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="b">
@@ -1223,10 +1223,10 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>21.7255</v>
+        <v>20.5945</v>
       </c>
       <c r="H14" t="n">
-        <v>1.177898047312858e-104</v>
+        <v>3.072222260418813e-94</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="b">
@@ -1253,10 +1253,10 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>-19.3202</v>
+        <v>-19.0566</v>
       </c>
       <c r="H15" t="n">
-        <v>3.634916082210407e-83</v>
+        <v>5.797086448503029e-81</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="b">

</xml_diff>